<commit_message>
Add AvaloniaXpfDrawingOptions and shared drawing logic
Introduced DrawingOptions.Shared project for cross-platform drawing logic and constants, now used by both WpfDrawingOptions and the new AvaloniaXpfDrawingOptions (Avalonia XPF) project. Refactored drawing controls and FrameRateMonitor to shared code, updated project/solution files, and added nuget.config for XPF feed. Also included Drawing Performance Comparisons.xlsx for benchmarking.
</commit_message>
<xml_diff>
--- a/Drawing Performance Comparisons.xlsx
+++ b/Drawing Performance Comparisons.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\WpfDrawingOptions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autonomoussolutions-my.sharepoint.com/personal/0194_asirobots_com/Documents/source/repos/WpfDrawingOptions/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33807CE8-EF7A-49BF-A39E-10F5AB60D1A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11385" xr2:uid="{563D8AC9-4C7D-4D50-B9DD-B1DB98568A2D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="34776" windowHeight="21096" xr2:uid="{563D8AC9-4C7D-4D50-B9DD-B1DB98568A2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -283,9 +283,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -323,7 +323,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -429,7 +429,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -571,7 +571,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -580,21 +580,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A1ED2D-F98C-441D-9C65-453932F04A7A}">
   <dimension ref="A1:W25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.109375" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>14</v>
       </c>
@@ -659,7 +659,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D2" t="s">
         <v>1</v>
       </c>
@@ -688,7 +688,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D3" t="s">
         <v>6</v>
       </c>
@@ -717,7 +717,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D4" s="12" t="s">
         <v>28</v>
       </c>
@@ -738,7 +738,7 @@
       <c r="Q4" s="2"/>
       <c r="U4" s="2"/>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D5" s="9" t="s">
         <v>7</v>
       </c>
@@ -767,7 +767,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="C6" s="10" t="s">
         <v>31</v>
       </c>
@@ -799,7 +799,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D7" s="9" t="s">
         <v>9</v>
       </c>
@@ -828,7 +828,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
         <v>10</v>
       </c>
@@ -857,7 +857,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
         <v>12</v>
       </c>
@@ -878,7 +878,7 @@
       <c r="Q9" s="2"/>
       <c r="U9" s="2"/>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="10">
         <v>4</v>
       </c>
@@ -943,7 +943,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="10">
         <v>3</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="11">
         <v>1</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
         <v>2</v>
       </c>
@@ -1138,7 +1138,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="10">
         <v>5</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="C16" s="10" t="s">
         <v>27</v>
       </c>
@@ -1211,42 +1211,42 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
       <c r="D17" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
       <c r="D18" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
       <c r="D20" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:4" x14ac:dyDescent="0.3">
       <c r="D21" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.3">
       <c r="D22" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:4" x14ac:dyDescent="0.3">
       <c r="D23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C25" s="10" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Add AvaloniaDrawingOptions project for drawing benchmarks
Introduces a new Avalonia UI project, AvaloniaDrawingOptions, to the solution. This project implements Avalonia equivalents for all WPF drawing benchmark modes, including DrawingVisual, Canvas, StreamGeometry, Skia (bitmap and direct), WriteableBitmap, and Composition API. The main window allows switching between drawing methods and running automated benchmarks, reporting frame and draw rates for each. Solution and project files updated accordingly; no changes to WPF or shared code. Also updates the Excel results file to reflect new Avalonia benchmarks.
</commit_message>
<xml_diff>
--- a/Drawing Performance Comparisons.xlsx
+++ b/Drawing Performance Comparisons.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autonomoussolutions-my.sharepoint.com/personal/0194_asirobots_com/Documents/source/repos/WpfDrawingOptions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eli.Taylor\OneDrive - ASI Robots\source\repos\WpfDrawingOptions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33807CE8-EF7A-49BF-A39E-10F5AB60D1A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B29CF5-9C6E-418B-847C-D1DFF66EDC73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="34776" windowHeight="21096" xr2:uid="{563D8AC9-4C7D-4D50-B9DD-B1DB98568A2D}"/>
+    <workbookView xWindow="28290" yWindow="-18840" windowWidth="25920" windowHeight="15360" xr2:uid="{563D8AC9-4C7D-4D50-B9DD-B1DB98568A2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Pure Avalonia" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="55">
   <si>
     <t>Technology</t>
   </si>
@@ -144,6 +145,63 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>Avalonia Drawing Visual</t>
+  </si>
+  <si>
+    <t>Avalonia Drawing Canvas</t>
+  </si>
+  <si>
+    <t>Avalonia Stream Geometry</t>
+  </si>
+  <si>
+    <t>Drawing Area</t>
+  </si>
+  <si>
+    <t>FR 5k</t>
+  </si>
+  <si>
+    <t>DR 5k</t>
+  </si>
+  <si>
+    <t>FR 25k</t>
+  </si>
+  <si>
+    <t>DR 25k</t>
+  </si>
+  <si>
+    <t>FR 50k</t>
+  </si>
+  <si>
+    <t>DR 50k</t>
+  </si>
+  <si>
+    <t>FR 100k</t>
+  </si>
+  <si>
+    <t>DR 100k</t>
+  </si>
+  <si>
+    <t>800x388</t>
+  </si>
+  <si>
+    <t>2304x1307</t>
+  </si>
+  <si>
+    <t>Pure Avalonia 800x388 px</t>
+  </si>
+  <si>
+    <t>Skia (Bitmap)</t>
+  </si>
+  <si>
+    <t>Direct Skia</t>
+  </si>
+  <si>
+    <t>Skia (WriteableBitmap)</t>
+  </si>
+  <si>
+    <t>Composition</t>
   </si>
 </sst>
 </file>
@@ -579,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A1ED2D-F98C-441D-9C65-453932F04A7A}">
-  <dimension ref="A1:W25"/>
+  <dimension ref="A1:W34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="10" bestFit="1" customWidth="1"/>
@@ -1211,47 +1269,581 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D17" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D18" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D20" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D21" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D22" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:19" x14ac:dyDescent="0.3">
       <c r="C25" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D25" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D27" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D28" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28">
+        <v>5000</v>
+      </c>
+      <c r="F28">
+        <v>29.2</v>
+      </c>
+      <c r="G28">
+        <v>29.6</v>
+      </c>
+      <c r="I28">
+        <v>25000</v>
+      </c>
+      <c r="J28">
+        <v>6.1</v>
+      </c>
+      <c r="K28">
+        <v>6.2</v>
+      </c>
+      <c r="M28">
+        <v>50000</v>
+      </c>
+      <c r="N28">
+        <v>2.7</v>
+      </c>
+      <c r="O28">
+        <v>2.7</v>
+      </c>
+      <c r="Q28">
+        <v>100000</v>
+      </c>
+      <c r="R28">
+        <v>1.6</v>
+      </c>
+      <c r="S28">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="29" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D29" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29">
+        <v>5000</v>
+      </c>
+      <c r="F29">
+        <v>30.1</v>
+      </c>
+      <c r="G29">
+        <v>30.4</v>
+      </c>
+      <c r="I29">
+        <v>25000</v>
+      </c>
+      <c r="J29">
+        <v>6.5</v>
+      </c>
+      <c r="K29">
+        <v>6.8</v>
+      </c>
+      <c r="M29">
+        <v>50000</v>
+      </c>
+      <c r="N29">
+        <v>3.1</v>
+      </c>
+      <c r="O29">
+        <v>3.2</v>
+      </c>
+      <c r="Q29">
+        <v>100000</v>
+      </c>
+      <c r="R29">
+        <v>1.5</v>
+      </c>
+      <c r="S29">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="30" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E30">
+        <v>5000</v>
+      </c>
+      <c r="F30">
+        <v>55.9</v>
+      </c>
+      <c r="G30">
+        <v>56</v>
+      </c>
+      <c r="I30">
+        <v>25000</v>
+      </c>
+      <c r="J30">
+        <v>1</v>
+      </c>
+      <c r="K30">
+        <v>2.1</v>
+      </c>
+      <c r="M30">
+        <v>50000</v>
+      </c>
+      <c r="N30">
+        <v>0.3</v>
+      </c>
+      <c r="O30">
+        <v>12.7</v>
+      </c>
+      <c r="Q30">
+        <v>100000</v>
+      </c>
+      <c r="R30">
+        <v>0.1</v>
+      </c>
+      <c r="S30">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="31" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D31" t="s">
+        <v>51</v>
+      </c>
+      <c r="E31">
+        <v>5000</v>
+      </c>
+      <c r="F31">
+        <v>7.9</v>
+      </c>
+      <c r="G31">
+        <v>7.9</v>
+      </c>
+      <c r="I31">
+        <v>25000</v>
+      </c>
+      <c r="J31">
+        <v>3.4</v>
+      </c>
+      <c r="K31">
+        <v>3.4</v>
+      </c>
+      <c r="M31">
+        <v>50000</v>
+      </c>
+      <c r="N31">
+        <v>2.1</v>
+      </c>
+      <c r="O31">
+        <v>2.1</v>
+      </c>
+      <c r="Q31">
+        <v>100000</v>
+      </c>
+      <c r="R31">
+        <v>0.1</v>
+      </c>
+      <c r="S31">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D32" t="s">
+        <v>52</v>
+      </c>
+      <c r="E32">
+        <v>5000</v>
+      </c>
+      <c r="F32">
+        <v>58.8</v>
+      </c>
+      <c r="G32">
+        <v>59.4</v>
+      </c>
+      <c r="I32">
+        <v>25000</v>
+      </c>
+      <c r="J32">
+        <v>15.1</v>
+      </c>
+      <c r="K32">
+        <v>15.8</v>
+      </c>
+      <c r="M32">
+        <v>50000</v>
+      </c>
+      <c r="N32">
+        <v>8.6</v>
+      </c>
+      <c r="O32">
+        <v>9.1</v>
+      </c>
+      <c r="Q32">
+        <v>100000</v>
+      </c>
+      <c r="R32">
+        <v>4.5</v>
+      </c>
+      <c r="S32">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="33" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+      <c r="E33">
+        <v>5000</v>
+      </c>
+      <c r="F33">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="G33">
+        <v>20.2</v>
+      </c>
+      <c r="I33">
+        <v>25000</v>
+      </c>
+      <c r="J33">
+        <v>4.8</v>
+      </c>
+      <c r="K33">
+        <v>4.8</v>
+      </c>
+      <c r="M33">
+        <v>50000</v>
+      </c>
+      <c r="N33">
+        <v>2.5</v>
+      </c>
+      <c r="O33">
+        <v>2.5</v>
+      </c>
+      <c r="Q33">
+        <v>100000</v>
+      </c>
+      <c r="R33">
+        <v>1.4</v>
+      </c>
+      <c r="S33">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="34" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E34">
+        <v>5000</v>
+      </c>
+      <c r="F34">
+        <v>49.8</v>
+      </c>
+      <c r="G34">
+        <v>50.7</v>
+      </c>
+      <c r="I34">
+        <v>25000</v>
+      </c>
+      <c r="J34">
+        <v>14.9</v>
+      </c>
+      <c r="K34">
+        <v>15</v>
+      </c>
+      <c r="M34">
+        <v>50000</v>
+      </c>
+      <c r="N34">
+        <v>8.5</v>
+      </c>
+      <c r="O34">
+        <v>8.6</v>
+      </c>
+      <c r="Q34">
+        <v>100000</v>
+      </c>
+      <c r="R34">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="S34">
+        <v>4.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C23B835A-8946-461F-B11D-76E21B3197AB}">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.6640625" customWidth="1"/>
+    <col min="5" max="7" width="9.77734375" customWidth="1"/>
+    <col min="8" max="9" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2">
+        <v>30.6</v>
+      </c>
+      <c r="D2">
+        <v>30.2</v>
+      </c>
+      <c r="E2">
+        <v>6.5</v>
+      </c>
+      <c r="F2">
+        <v>6.6</v>
+      </c>
+      <c r="G2">
+        <v>3.3</v>
+      </c>
+      <c r="H2">
+        <v>3.4</v>
+      </c>
+      <c r="I2">
+        <v>1.6</v>
+      </c>
+      <c r="J2">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3">
+        <v>24.7</v>
+      </c>
+      <c r="D3">
+        <v>25.1</v>
+      </c>
+      <c r="E3">
+        <v>5.9</v>
+      </c>
+      <c r="F3">
+        <v>6.2</v>
+      </c>
+      <c r="G3">
+        <v>3.1</v>
+      </c>
+      <c r="H3">
+        <v>3.3</v>
+      </c>
+      <c r="I3">
+        <v>1.6</v>
+      </c>
+      <c r="J3">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4">
+        <v>29.5</v>
+      </c>
+      <c r="D4">
+        <v>29.5</v>
+      </c>
+      <c r="E4">
+        <v>6.5</v>
+      </c>
+      <c r="F4">
+        <v>6.7</v>
+      </c>
+      <c r="G4">
+        <v>3.3</v>
+      </c>
+      <c r="H4">
+        <v>3.4</v>
+      </c>
+      <c r="I4">
+        <v>1.7</v>
+      </c>
+      <c r="J4">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5">
+        <v>26.1</v>
+      </c>
+      <c r="D5">
+        <v>25.6</v>
+      </c>
+      <c r="E5">
+        <v>5.7</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="G5">
+        <v>2.7</v>
+      </c>
+      <c r="H5">
+        <v>2.8</v>
+      </c>
+      <c r="I5">
+        <v>1.5</v>
+      </c>
+      <c r="J5">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6">
+        <v>57.3</v>
+      </c>
+      <c r="D6">
+        <v>57.6</v>
+      </c>
+      <c r="E6">
+        <v>1.9</v>
+      </c>
+      <c r="F6">
+        <v>2.5</v>
+      </c>
+      <c r="G6">
+        <v>0.3</v>
+      </c>
+      <c r="H6">
+        <v>2.7</v>
+      </c>
+      <c r="I6">
+        <v>0.1</v>
+      </c>
+      <c r="J6">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7">
+        <v>3.9</v>
+      </c>
+      <c r="D7">
+        <v>4.5</v>
+      </c>
+      <c r="E7">
+        <v>0.4</v>
+      </c>
+      <c r="F7">
+        <v>7.7</v>
+      </c>
+      <c r="G7">
+        <v>0.1</v>
+      </c>
+      <c r="H7">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>1.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Drawing Performance Comparisons.xlsx data
The Excel spreadsheet was updated with new or revised data,
reflecting changes in drawing performance comparisons. No
code changes were made.
</commit_message>
<xml_diff>
--- a/Drawing Performance Comparisons.xlsx
+++ b/Drawing Performance Comparisons.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://autonomoussolutions-my.sharepoint.com/personal/0194_asirobots_com/Documents/source/repos/WpfDrawingOptions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eli.Taylor\OneDrive - ASI Robots\source\repos\WpfDrawingOptions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33807CE8-EF7A-49BF-A39E-10F5AB60D1A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B29CF5-9C6E-418B-847C-D1DFF66EDC73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="34776" windowHeight="21096" xr2:uid="{563D8AC9-4C7D-4D50-B9DD-B1DB98568A2D}"/>
+    <workbookView xWindow="28290" yWindow="-18840" windowWidth="25920" windowHeight="15360" xr2:uid="{563D8AC9-4C7D-4D50-B9DD-B1DB98568A2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Pure Avalonia" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="55">
   <si>
     <t>Technology</t>
   </si>
@@ -144,6 +145,63 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>Avalonia Drawing Visual</t>
+  </si>
+  <si>
+    <t>Avalonia Drawing Canvas</t>
+  </si>
+  <si>
+    <t>Avalonia Stream Geometry</t>
+  </si>
+  <si>
+    <t>Drawing Area</t>
+  </si>
+  <si>
+    <t>FR 5k</t>
+  </si>
+  <si>
+    <t>DR 5k</t>
+  </si>
+  <si>
+    <t>FR 25k</t>
+  </si>
+  <si>
+    <t>DR 25k</t>
+  </si>
+  <si>
+    <t>FR 50k</t>
+  </si>
+  <si>
+    <t>DR 50k</t>
+  </si>
+  <si>
+    <t>FR 100k</t>
+  </si>
+  <si>
+    <t>DR 100k</t>
+  </si>
+  <si>
+    <t>800x388</t>
+  </si>
+  <si>
+    <t>2304x1307</t>
+  </si>
+  <si>
+    <t>Pure Avalonia 800x388 px</t>
+  </si>
+  <si>
+    <t>Skia (Bitmap)</t>
+  </si>
+  <si>
+    <t>Direct Skia</t>
+  </si>
+  <si>
+    <t>Skia (WriteableBitmap)</t>
+  </si>
+  <si>
+    <t>Composition</t>
   </si>
 </sst>
 </file>
@@ -579,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A1ED2D-F98C-441D-9C65-453932F04A7A}">
-  <dimension ref="A1:W25"/>
+  <dimension ref="A1:W34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="10" bestFit="1" customWidth="1"/>
@@ -1211,47 +1269,581 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D17" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D18" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D20" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D21" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D22" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:19" x14ac:dyDescent="0.3">
       <c r="D23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:19" x14ac:dyDescent="0.3">
       <c r="C25" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D25" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D27" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D28" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28">
+        <v>5000</v>
+      </c>
+      <c r="F28">
+        <v>29.2</v>
+      </c>
+      <c r="G28">
+        <v>29.6</v>
+      </c>
+      <c r="I28">
+        <v>25000</v>
+      </c>
+      <c r="J28">
+        <v>6.1</v>
+      </c>
+      <c r="K28">
+        <v>6.2</v>
+      </c>
+      <c r="M28">
+        <v>50000</v>
+      </c>
+      <c r="N28">
+        <v>2.7</v>
+      </c>
+      <c r="O28">
+        <v>2.7</v>
+      </c>
+      <c r="Q28">
+        <v>100000</v>
+      </c>
+      <c r="R28">
+        <v>1.6</v>
+      </c>
+      <c r="S28">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="29" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D29" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29">
+        <v>5000</v>
+      </c>
+      <c r="F29">
+        <v>30.1</v>
+      </c>
+      <c r="G29">
+        <v>30.4</v>
+      </c>
+      <c r="I29">
+        <v>25000</v>
+      </c>
+      <c r="J29">
+        <v>6.5</v>
+      </c>
+      <c r="K29">
+        <v>6.8</v>
+      </c>
+      <c r="M29">
+        <v>50000</v>
+      </c>
+      <c r="N29">
+        <v>3.1</v>
+      </c>
+      <c r="O29">
+        <v>3.2</v>
+      </c>
+      <c r="Q29">
+        <v>100000</v>
+      </c>
+      <c r="R29">
+        <v>1.5</v>
+      </c>
+      <c r="S29">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="30" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E30">
+        <v>5000</v>
+      </c>
+      <c r="F30">
+        <v>55.9</v>
+      </c>
+      <c r="G30">
+        <v>56</v>
+      </c>
+      <c r="I30">
+        <v>25000</v>
+      </c>
+      <c r="J30">
+        <v>1</v>
+      </c>
+      <c r="K30">
+        <v>2.1</v>
+      </c>
+      <c r="M30">
+        <v>50000</v>
+      </c>
+      <c r="N30">
+        <v>0.3</v>
+      </c>
+      <c r="O30">
+        <v>12.7</v>
+      </c>
+      <c r="Q30">
+        <v>100000</v>
+      </c>
+      <c r="R30">
+        <v>0.1</v>
+      </c>
+      <c r="S30">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="31" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D31" t="s">
+        <v>51</v>
+      </c>
+      <c r="E31">
+        <v>5000</v>
+      </c>
+      <c r="F31">
+        <v>7.9</v>
+      </c>
+      <c r="G31">
+        <v>7.9</v>
+      </c>
+      <c r="I31">
+        <v>25000</v>
+      </c>
+      <c r="J31">
+        <v>3.4</v>
+      </c>
+      <c r="K31">
+        <v>3.4</v>
+      </c>
+      <c r="M31">
+        <v>50000</v>
+      </c>
+      <c r="N31">
+        <v>2.1</v>
+      </c>
+      <c r="O31">
+        <v>2.1</v>
+      </c>
+      <c r="Q31">
+        <v>100000</v>
+      </c>
+      <c r="R31">
+        <v>0.1</v>
+      </c>
+      <c r="S31">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="3:19" x14ac:dyDescent="0.3">
+      <c r="D32" t="s">
+        <v>52</v>
+      </c>
+      <c r="E32">
+        <v>5000</v>
+      </c>
+      <c r="F32">
+        <v>58.8</v>
+      </c>
+      <c r="G32">
+        <v>59.4</v>
+      </c>
+      <c r="I32">
+        <v>25000</v>
+      </c>
+      <c r="J32">
+        <v>15.1</v>
+      </c>
+      <c r="K32">
+        <v>15.8</v>
+      </c>
+      <c r="M32">
+        <v>50000</v>
+      </c>
+      <c r="N32">
+        <v>8.6</v>
+      </c>
+      <c r="O32">
+        <v>9.1</v>
+      </c>
+      <c r="Q32">
+        <v>100000</v>
+      </c>
+      <c r="R32">
+        <v>4.5</v>
+      </c>
+      <c r="S32">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="33" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+      <c r="E33">
+        <v>5000</v>
+      </c>
+      <c r="F33">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="G33">
+        <v>20.2</v>
+      </c>
+      <c r="I33">
+        <v>25000</v>
+      </c>
+      <c r="J33">
+        <v>4.8</v>
+      </c>
+      <c r="K33">
+        <v>4.8</v>
+      </c>
+      <c r="M33">
+        <v>50000</v>
+      </c>
+      <c r="N33">
+        <v>2.5</v>
+      </c>
+      <c r="O33">
+        <v>2.5</v>
+      </c>
+      <c r="Q33">
+        <v>100000</v>
+      </c>
+      <c r="R33">
+        <v>1.4</v>
+      </c>
+      <c r="S33">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="34" spans="4:19" x14ac:dyDescent="0.3">
+      <c r="D34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E34">
+        <v>5000</v>
+      </c>
+      <c r="F34">
+        <v>49.8</v>
+      </c>
+      <c r="G34">
+        <v>50.7</v>
+      </c>
+      <c r="I34">
+        <v>25000</v>
+      </c>
+      <c r="J34">
+        <v>14.9</v>
+      </c>
+      <c r="K34">
+        <v>15</v>
+      </c>
+      <c r="M34">
+        <v>50000</v>
+      </c>
+      <c r="N34">
+        <v>8.5</v>
+      </c>
+      <c r="O34">
+        <v>8.6</v>
+      </c>
+      <c r="Q34">
+        <v>100000</v>
+      </c>
+      <c r="R34">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="S34">
+        <v>4.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C23B835A-8946-461F-B11D-76E21B3197AB}">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.6640625" customWidth="1"/>
+    <col min="5" max="7" width="9.77734375" customWidth="1"/>
+    <col min="8" max="9" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2">
+        <v>30.6</v>
+      </c>
+      <c r="D2">
+        <v>30.2</v>
+      </c>
+      <c r="E2">
+        <v>6.5</v>
+      </c>
+      <c r="F2">
+        <v>6.6</v>
+      </c>
+      <c r="G2">
+        <v>3.3</v>
+      </c>
+      <c r="H2">
+        <v>3.4</v>
+      </c>
+      <c r="I2">
+        <v>1.6</v>
+      </c>
+      <c r="J2">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3">
+        <v>24.7</v>
+      </c>
+      <c r="D3">
+        <v>25.1</v>
+      </c>
+      <c r="E3">
+        <v>5.9</v>
+      </c>
+      <c r="F3">
+        <v>6.2</v>
+      </c>
+      <c r="G3">
+        <v>3.1</v>
+      </c>
+      <c r="H3">
+        <v>3.3</v>
+      </c>
+      <c r="I3">
+        <v>1.6</v>
+      </c>
+      <c r="J3">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4">
+        <v>29.5</v>
+      </c>
+      <c r="D4">
+        <v>29.5</v>
+      </c>
+      <c r="E4">
+        <v>6.5</v>
+      </c>
+      <c r="F4">
+        <v>6.7</v>
+      </c>
+      <c r="G4">
+        <v>3.3</v>
+      </c>
+      <c r="H4">
+        <v>3.4</v>
+      </c>
+      <c r="I4">
+        <v>1.7</v>
+      </c>
+      <c r="J4">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5">
+        <v>26.1</v>
+      </c>
+      <c r="D5">
+        <v>25.6</v>
+      </c>
+      <c r="E5">
+        <v>5.7</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="G5">
+        <v>2.7</v>
+      </c>
+      <c r="H5">
+        <v>2.8</v>
+      </c>
+      <c r="I5">
+        <v>1.5</v>
+      </c>
+      <c r="J5">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6">
+        <v>57.3</v>
+      </c>
+      <c r="D6">
+        <v>57.6</v>
+      </c>
+      <c r="E6">
+        <v>1.9</v>
+      </c>
+      <c r="F6">
+        <v>2.5</v>
+      </c>
+      <c r="G6">
+        <v>0.3</v>
+      </c>
+      <c r="H6">
+        <v>2.7</v>
+      </c>
+      <c r="I6">
+        <v>0.1</v>
+      </c>
+      <c r="J6">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7">
+        <v>3.9</v>
+      </c>
+      <c r="D7">
+        <v>4.5</v>
+      </c>
+      <c r="E7">
+        <v>0.4</v>
+      </c>
+      <c r="F7">
+        <v>7.7</v>
+      </c>
+      <c r="G7">
+        <v>0.1</v>
+      </c>
+      <c r="H7">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>1.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>